<commit_message>
data: 2026-07-22 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-07/2026-07-22.xlsx
+++ b/data/daily/2026-07/2026-07-22.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리통계" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="올리브영" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="카카오선물하기" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="다이소몰" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="올리브영" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="카테고리통계" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -902,22 +902,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
+          <t>아르기닌 증정 남친 활력선물 대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>48,900원</t>
+          <t>45,000원</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11566779</t>
+          <t>https://gift.kakao.com/product/7417420</t>
         </is>
       </c>
     </row>
@@ -932,22 +932,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>아르기닌 증정 남친 활력선물 대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
+          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>익스트림</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>45,000원</t>
+          <t>19,900원</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7417420</t>
+          <t>https://gift.kakao.com/product/10848340</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
+          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>19,900원</t>
+          <t>48,900원</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/10848340</t>
+          <t>https://gift.kakao.com/product/11566779</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>61,900원</t>
+          <t>65,900원</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1022,29 +1022,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>카카오 단독제품 '선물하기 단독' 완전균형영양식 간편한끼 뉴케어 구수한맛 7입+오트아몬드 7입 14개입(1BOX)</t>
+          <t>아메리카노 증정 에너지 활력선물 [김종국 추천세트]익스트림 아르기닌정 (2개월분) &amp; 밀크씨슬 플러스 (2개월분) + 쇼핑백 증정</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>뉴케어</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>32,900원</t>
+          <t>25,900원</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/13688976</t>
+          <t>https://gift.kakao.com/product/7556791</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1052,22 +1052,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)</t>
+          <t>[운동선물/헬스] 삼대오백 모노 크레아틴 100서빙 운동 필수템 +키링증정</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>그레인온</t>
+          <t>삼대오백</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>24,900원</t>
+          <t>17,900원</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/13180362</t>
+          <t>https://gift.kakao.com/product/6352718</t>
         </is>
       </c>
     </row>
@@ -1085,10 +1085,10 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1128,7 +1128,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1136,12 +1136,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>토비콤 눈피로엔 아이포커스 미니 20캡슐</t>
+          <t>멀티비타민 미네랄 30정 30일분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>안국약품</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1151,14 +1151,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=611982832&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000135&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>비타민C/항산화</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1166,29 +1166,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>리포좀 비타민C 30정</t>
+          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910679&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>바나바잎 추출물 30정 (30일분)</t>
+          <t>마그네슘 30정 30일분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000131&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>콜린 미오이노시톨 4000 10포</t>
+          <t>푸응 7days 팻버닝 21캡슐</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>안국약품</t>
+          <t>닥터블릿</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1241,14 +1241,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=985472642&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602085&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1256,22 +1256,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>데일리와이즈 초임계 알티지 오메가3 12캡슐 12일분</t>
+          <t>녹차 카테킨 6정 6일분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>종근당</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>1,000원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032306203&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000282&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1286,12 +1286,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>밀크씨슬 30정 30일분</t>
+          <t>콜린 미오이노시톨 4000 10포</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>안국약품</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1301,14 +1301,14 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000134&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=985472642&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1316,29 +1316,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>철분 30정 30일분</t>
+          <t>LG생활건강 이너뷰 콜라겐 더마스틱 7포</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>이너뷰 바이 리튠</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000133&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=994953528&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1346,29 +1346,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>코엔자임 Q10 30캡슐 30일분</t>
+          <t>동화 부채표 편안활 5포 5일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동화약품</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=601618636&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>눈건강엔 루테인지아잔틴</t>
+          <t>더채움 비오틴 하루구미 30일분</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>종근당건강</t>
+          <t>오브맘</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1391,14 +1391,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=591580541&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=613602127&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1406,22 +1406,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>데일리와이즈 코엔자임Q10 12캡슐 12일분</t>
+          <t>유기농 엑스트라버진 올리브유 10포</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>종근당</t>
+          <t>홀베리</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032306202&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032640075&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1431,6 +1431,320 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>순위</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>상품명</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>가격</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>비비랩 슬림 밸런스 유산균 2g x 30포 (15일분)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>비비랩</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>18,900원</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>비비랩 데일리 밸런스 유산균 2g x 30포 (1개월분)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>비비랩</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>16,900원</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>다이어트/체중관리</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>프로뉴트리션</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>35,800원</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>피부/미용</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[7월 올영픽/단독기획] 비비랩 저분자콜라겐S 30포 단품/더블기획</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>비비랩</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>26,900원</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>비타민C/항산화</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>고려은단 비타민C1000 600정 (20개월분)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>고려은단</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>42,900원</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[7월 올영픽] 콜레올로직 컷팅 젤리 레몬/키위/석류 10+2+2포 기획</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>푸드올로지</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>18,800원</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>올더베리 웰니스 구미 30일분 6종 택1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>올더베리</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>9,500원</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>기타/특수목적</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[골라담기] CJ웰케어 건강루틴 10종 택1 가격혁명</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>씨제이웰케어</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5,900원</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[올영단독] 지노마스터 질유산균 70캡슐 (70일분)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>지노마스터</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>59,000원</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>프로바이오틱스/유산균</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균)+철분 헤모케어3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>덴프스</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>39,000원</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1448,32 +1762,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1486,16 +1800,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="D2" t="n">
         <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1508,16 +1822,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
@@ -1552,16 +1866,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1574,16 +1888,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -1596,16 +1910,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1640,13 +1954,13 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" t="n">
         <v>6</v>
-      </c>
-      <c r="C9" t="n">
-        <v>15</v>
-      </c>
-      <c r="D9" t="n">
-        <v>4</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -1684,16 +1998,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -1706,16 +2020,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
@@ -1742,320 +2056,6 @@
       <c r="F13" t="n">
         <v>10</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>카테고리</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>순위</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>상품명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>가격</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>상품URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>프로바이오틱스/유산균</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>비비랩 슬림 밸런스 유산균 2g x 30포 (15일분)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>비비랩</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>18,900원</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>프로바이오틱스/유산균</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>비비랩 데일리 밸런스 유산균 2g x 30포 (1개월분)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>비비랩</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>16,900원</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>다이어트/체중관리</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>프로뉴트리션</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>35,800원</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>피부/미용</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>[7월 올영픽/단독기획] 비비랩 저분자콜라겐S 30포 단품/더블기획</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>비비랩</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>26,900원</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>비타민C/항산화</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>고려은단 비타민C1000 600정 (20개월분)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>고려은단</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>42,900원</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>[7월 올영픽] 콜레올로직 컷팅 젤리 레몬/키위/석류 10+2+2포 기획</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>푸드올로지</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>18,800원</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>올더베리 웰니스 구미 30일분 6종 택1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>올더베리</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>9,500원</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>기타/특수목적</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>[골라담기] CJ웰케어 건강루틴 10종 택1 가격혁명</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>씨제이웰케어</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>5,900원</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>프로바이오틱스/유산균</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>[올영단독] 지노마스터 질유산균 70캡슐 (70일분)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>지노마스터</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>59,000원</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>프로바이오틱스/유산균</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균)+철분 헤모케어3</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>덴프스</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>39,000원</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>